<commit_message>
Update to allow the pipeline to run normally, require bugfix in ui + how to extract paper + returned table
</commit_message>
<xml_diff>
--- a/table_from_link/30448613_table1.xlsx
+++ b/table_from_link/30448613_table1.xlsx
@@ -413,315 +413,331 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>IGAP SNP | SNP | SNP</t>
+          <t>IGAP SNP</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>IGAP SNP | Closest gene | Closest gene</t>
+          <t>IGAP SNP</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>IGAP SNP | ADGC a | OR</t>
+          <t>IGAP SNP</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>IGAP SNP | ADGC a | P-value</t>
+          <t>IGAP SNP</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Exonic SNP | SNP ID | SNP ID</t>
+          <t>Exonic SNP</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Exonic SNP | ADGC a | OR</t>
+          <t>Exonic SNP</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Exonic SNP | ADGC a | P-value</t>
+          <t>Exonic SNP</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Exonic SNP | ADSP b | OR</t>
+          <t>Exonic SNP</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Exonic SNP | ADSP b | P-value</t>
+          <t>Exonic SNP</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>SNP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>Closest gene</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>ADGC a</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>ADGC a</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>SNP ID</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>ADGC a</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>ADGC a</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>ADSP b</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Strong LD (r2 ≥ 0.8)</t>
+          <t>ADSP b</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rs6656401</t>
+          <t>SNP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CR1</t>
+          <t>Closest gene</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8.49 ×10−7</t>
+          <t>P-value</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>rs4844600</t>
+          <t>SNP ID</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4.22×10−7</t>
+          <t>P-value</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>P-value</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>rs2296160</t>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4.24×10−8</t>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>8.56×10−3</t>
+          <t>Strong LD (r 2 ≥ 0.8)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>rs6656401</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CR1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8.49 ×10 −7</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>rs4844600</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>4.22×10 −7</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>rs2296160</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>4.24×10 −8</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>8.56×10 −3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>rs9271192</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>HLA-DRB5</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>1.11</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2.66×10−4</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2.66×10 −4</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>rs9270303</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>1.15</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2.50×10−4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>rs1476679</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ZCWPW1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0.92</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1.41×10−3</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>rs2405442</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>0.92</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2.12×10−3</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>0.89</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>1.09×10−3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>rs1859788</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.93</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>5.62×10−3</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.89</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.12×10−3</t>
+          <t>2.50×10 −4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rs9331896</t>
+          <t>rs1476679</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -731,218 +747,296 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.02×10−3</t>
+          <t>1.41×10 −3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>rs7982</t>
+          <t>rs2405442</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3.64×10−4</t>
+          <t>2.12×10 −3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.62×10−3</t>
+          <t>1.09×10 −3</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>rs10838725</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CELF1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1.05</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>0.054</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>rs2293576</t>
+          <t>rs1859788</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>5.62×10 −3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.040</t>
+          <t>1.12×10 −3</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rs983392</t>
+          <t>rs9331896</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7.22×10−9</t>
+          <t>1.02×10 −3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>rs12453</t>
+          <t>rs7982</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.34×10−9</t>
+          <t>3.64×10 −4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3.60×10−4</t>
+          <t>1.62×10 −3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rs4147929</t>
+          <t>rs10838725</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.39×10−3</t>
+          <t>0.054</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>rs3752246</t>
+          <t>rs2293576</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2.70×10−3</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>9.89×10−5</t>
+          <t>0.040</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>rs983392</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MS4A6A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>7.22×10 −9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>rs12453</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1.34×10 −9</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.89</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3.60×10 −4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>rs4147929</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1.39×10 −3</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>rs3752246</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2.70×10 −3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>9.89×10 −5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>rs3865444</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>CD33</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>0.91</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>4.49 ×10−4</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4.49 ×10 −4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>rs12459419</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>0.91</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>4.02×10−4</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4.02×10 −4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>0.94</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>0.090</t>
         </is>

</xml_diff>